<commit_message>
Add Light Plant and Concrete Mixer to portable equipment (wet/dry day rates)
Five catalogue items appended after the Excel sheet items on every build,
via the new EXTRA_PORTABLE list in tools/build_fleet_data.py:
- Light Plant 4x400W LED tower (diesel): 9,500 / 6,000
- Light Plant 4x1000W metal-halide tower (diesel): 12,500 / 8,000
- Concrete Mixer 5/3.5 cu.ft petrol half-bag: 3,000 / 2,000
- Concrete Mixer 10/7 cu.ft diesel one-bag drum: 4,500 / 3,000
- Concrete Mixer 10/7 cu.ft with hopper/hoist: 6,500 / 4,500
Rates are Rs./day excl. VAT, WET = incl. fuel & operator, DRY = bare hire.
Rate-card Excel regenerated; tests updated (41 portable items).

https://claude.ai/code/session_01S39wHpjtFMD4YJDii92yPt
</commit_message>
<xml_diff>
--- a/data/Fleet_Rental_Rate_Matrix_2026.xlsx
+++ b/data/Fleet_Rental_Rate_Matrix_2026.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fleet Rate Matrix'!$A$4:$R$522</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Portable Equipment'!$A$4:$E$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Portable Equipment'!$A$4:$E$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33111,7 +33111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -33918,8 +33918,113 @@
         <v>6500</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Light Plant</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>4×400 W LED tower (mobile, diesel)</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>9500</v>
+      </c>
+      <c r="E41" s="11" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Light Plant</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>4×1000 W metal-halide tower (diesel)</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>12500</v>
+      </c>
+      <c r="E42" s="11" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Concrete Mixer</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>5/3.5 cu.ft (petrol, half-bag)</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E43" s="11" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Concrete Mixer</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>10/7 cu.ft drum (diesel, one-bag)</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E44" s="11" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Concrete Mixer</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>10/7 cu.ft with hopper / hoist</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E45" s="11" t="n">
+        <v>4500</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E40"/>
+  <autoFilter ref="A4:E45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>